<commit_message>
Resolved merge conflicts and finalized code
</commit_message>
<xml_diff>
--- a/agent_4/output/Master_Database.xlsx
+++ b/agent_4/output/Master_Database.xlsx
@@ -533,7 +533,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>listing_4be6f6eee7554814</t>
+          <t>listing_4515d831654c4274</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tree Trimming &amp; Removal and Hedge Care</t>
+          <t>Semi-Passive Business: Predictable Profits</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>King County , WA</t>
+          <t>DeSoto County , MS</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -563,17 +563,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2000000</t>
+          <t>525000</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1300000</t>
+          <t>240000</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>250000</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://www.bizbuysell.com/business-opportunity/tree-trimming-and-removal-and-hedge-care/2460556/</t>
+          <t>https://www.bizbuysell.com/business-opportunity/semi-passive-business-predictable-profits/2460665/</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Gregory Kovsky</t>
+          <t>Dennis Anderson</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -602,10 +602,13 @@
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="P2">
+        <f>"+1-800-555-3699"</f>
+        <v/>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/all/?keywords=Gregory+Kovsky</t>
+          <t>https://www.linkedin.com/search/results/all/?keywords=Dennis+Anderson</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -615,7 +618,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>listing_26d595dc509243c8</t>
+          <t>listing_59261214ea2e428b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -630,12 +633,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Retail Stores Businesses for Sale</t>
+          <t>Business Service Businesses for Sale</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Duval County ,  Florida</t>
+          <t>Alameda County ,  California</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -645,12 +648,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1165000</t>
+          <t>700000</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1100000</t>
+          <t>497399</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -665,7 +668,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://www.bizquest.com/business-for-sale/established-full-service-sign-and-graphics-business/BW2460509/</t>
+          <t>https://www.bizquest.com/business-for-sale/100-occupied-salon-suite-for-sale-semi-absentee-model/BW2460616/</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -685,7 +688,7 @@
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3">
-        <f>"+1-561-676-1038"</f>
+        <f>"+1-210-970-7724"</f>
         <v/>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -696,7 +699,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>listing_189a60d9bd194b40</t>
+          <t>listing_d65edb0a8a70425f</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -771,7 +774,7 @@
         </is>
       </c>
       <c r="P4">
-        <f>"+1-800-613-1303"</f>
+        <f>"+1-888-770-7332"</f>
         <v/>
       </c>
       <c r="Q4" t="inlineStr">
@@ -781,26 +784,22 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Introduction: Acquisition Capital Partners &amp; Off-Market Real Estate Opportunities</t>
+          <t>Off-Market Opportunities - Acquisition Capital Partners</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Dear Mr. Zambito,
-My name is John Smith, and I am the Senior Acquisitions Manager at Acquisition Capital Partners. We are a well-capitalized investment firm actively seeking strategic real estate acquisitions across various asset classes. Our focus is on identifying and acquiring high-quality, income-producing, and value-add commercial properties.
-Our investment thesis is particularly strong for opportunities within the Park, PA region and broader Pennsylvania market. We are keen on properties that align with long-term growth potential and stable cash flow, demonstrating our commitment to thoughtful, strategic investments.
-Given J.C. BAR Properties, Inc.'s esteemed reputation and deep local market expertise, we are specifically interested in learning about any off-market opportunities or upcoming mandates that may fit our acquisition criteria. We value proprietary deal flow and believe our efficient due diligence process and certainty of close would be beneficial to your clients.
-I would appreciate the opportunity to schedule a brief call or meeting at your convenience to discuss our acquisition parameters in more detail and explore how we might collaborate on future transactions. Please let me know what time works best for you.
-Thank you for your time and consideration.
-Sincerely,
+          <t>Hi Pace,
+I'm John Smith from Acquisition Capital Partners. We are actively seeking off-market acquisition opportunities across various sectors for our clients. If you have any relevant deals that fit our criteria and are not publicly listed, please send them our way for immediate review. We're ready to move quickly on suitable opportunities.
+Thanks,
 John Smith
-Senior Acquisitions Manager
-Acquisition Capital Partners</t>
+Acquisition Capital Partners
+&lt;/email body&gt;</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>professional</t>
+          <t>direct</t>
         </is>
       </c>
     </row>

</xml_diff>